<commit_message>
sync: 2026-03-27 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
@@ -833,8 +833,8 @@
       <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>17</v>
+      <c r="C4" s="10" t="s">
+        <v>23</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>18</v>
@@ -870,7 +870,7 @@
         <v>0</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -934,7 +934,7 @@
         <v>35</v>
       </c>
       <c r="E6" s="8">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
sync: 2026-04-01 08:05 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="83">
   <si>
     <t>ID da Campanha</t>
   </si>
@@ -60,24 +60,36 @@
     <t>Observações</t>
   </si>
   <si>
+    <t>120245952608920204</t>
+  </si>
+  <si>
+    <t>[Syra] Aquecimento e Construção de Público [Vídeo Views] [ABO]</t>
+  </si>
+  <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>OUTCOME_ENGAGEMENT</t>
+  </si>
+  <si>
+    <t>31/03/2026</t>
+  </si>
+  <si>
+    <t>✅ Ativa</t>
+  </si>
+  <si>
     <t>120244701890430204</t>
   </si>
   <si>
     <t>[Syra] [Formulário Instantâneo] [ABO]</t>
   </si>
   <si>
-    <t>ACTIVE</t>
-  </si>
-  <si>
     <t>OUTCOME_LEADS</t>
   </si>
   <si>
     <t>04/03/2026</t>
   </si>
   <si>
-    <t>✅ Ativa</t>
-  </si>
-  <si>
     <t>120244387366780204</t>
   </si>
   <si>
@@ -118,9 +130,6 @@
   </si>
   <si>
     <t>[Syra] GERAR TOPO [Vídeo Views] [CBO]</t>
-  </si>
-  <si>
-    <t>OUTCOME_ENGAGEMENT</t>
   </si>
   <si>
     <t>120242992612760204</t>
@@ -666,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -786,14 +795,14 @@
       <c r="B3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
         <v>23</v>
       </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
       <c r="E3" s="1">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>24</v>
@@ -823,24 +832,24 @@
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E4" s="8">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>28</v>
@@ -870,24 +879,24 @@
         <v>0</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
       <c r="E5" s="1">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F5" t="s">
         <v>32</v>
@@ -917,7 +926,7 @@
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -927,17 +936,17 @@
       <c r="B6" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>17</v>
+      <c r="C6" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E6" s="8">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G6" s="6">
         <v>0</v>
@@ -964,27 +973,27 @@
         <v>0</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>23</v>
+        <v>38</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
       </c>
       <c r="E7" s="1">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1011,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1022,10 +1031,10 @@
         <v>40</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>23</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="E8" s="8">
         <v>0</v>
@@ -1058,7 +1067,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1069,10 +1078,10 @@
         <v>43</v>
       </c>
       <c r="C9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
         <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>35</v>
       </c>
       <c r="E9" s="1">
         <v>0</v>
@@ -1105,7 +1114,7 @@
         <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1116,13 +1125,13 @@
         <v>46</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E10" s="8">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>47</v>
@@ -1152,7 +1161,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1163,13 +1172,13 @@
         <v>49</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
         <v>18</v>
       </c>
       <c r="E11" s="1">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
         <v>50</v>
@@ -1199,7 +1208,7 @@
         <v>0</v>
       </c>
       <c r="O11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1210,10 +1219,10 @@
         <v>52</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>23</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="E12" s="8">
         <v>0</v>
@@ -1246,7 +1255,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1257,13 +1266,13 @@
         <v>55</v>
       </c>
       <c r="C13" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s">
         <v>23</v>
       </c>
-      <c r="D13" t="s">
-        <v>18</v>
-      </c>
       <c r="E13" s="1">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F13" t="s">
         <v>56</v>
@@ -1293,7 +1302,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1304,16 +1313,16 @@
         <v>58</v>
       </c>
       <c r="C14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E14" s="8">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G14" s="6">
         <v>0</v>
@@ -1340,28 +1349,28 @@
         <v>0</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="1">
+        <v>40</v>
+      </c>
+      <c r="F15" t="s">
         <v>59</v>
       </c>
-      <c r="B15" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E15" s="1">
-        <v>0</v>
-      </c>
-      <c r="F15" t="s">
-        <v>56</v>
-      </c>
       <c r="G15">
         <v>0</v>
       </c>
@@ -1387,27 +1396,27 @@
         <v>0</v>
       </c>
       <c r="O15" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>18</v>
-      </c>
       <c r="E16" s="8">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G16" s="6">
         <v>0</v>
@@ -1434,7 +1443,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -1445,13 +1454,13 @@
         <v>65</v>
       </c>
       <c r="C17" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" t="s">
         <v>23</v>
       </c>
-      <c r="D17" t="s">
-        <v>35</v>
-      </c>
       <c r="E17" s="1">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F17" t="s">
         <v>66</v>
@@ -1481,7 +1490,54 @@
         <v>0</v>
       </c>
       <c r="O17" t="s">
-        <v>25</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" s="8">
+        <v>10</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6">
+        <v>0</v>
+      </c>
+      <c r="I18" s="8">
+        <v>0</v>
+      </c>
+      <c r="J18" s="8">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
+        <v>0</v>
+      </c>
+      <c r="M18" s="9">
+        <v>0</v>
+      </c>
+      <c r="N18" s="8">
+        <v>0</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1510,13 +1566,13 @@
   <sheetData>
     <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -1525,7 +1581,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
@@ -1540,30 +1596,30 @@
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1581,7 +1637,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1608,19 +1664,19 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -1638,24 +1694,24 @@
         <v>2</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1670,10 +1726,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync: 2026-04-02 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
@@ -129,7 +129,7 @@
     <t>120243269097920204</t>
   </si>
   <si>
-    <t>[Syra] GERAR TOPO [Vídeo Views] [CBO]</t>
+    <t>[Syra] GERAR TOPO [Visita ao Perfil] [CBO]</t>
   </si>
   <si>
     <t>120242992612760204</t>
@@ -990,7 +990,7 @@
         <v>18</v>
       </c>
       <c r="E7" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
sync: 2026-04-06 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
@@ -983,8 +983,8 @@
       <c r="B7" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>17</v>
+      <c r="C7" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
sync: 2026-04-07 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-erico-servano/campaigns/data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="81">
   <si>
     <t>ID da Campanha</t>
   </si>
@@ -66,7 +66,7 @@
     <t>[Syra] Aquecimento e Construção de Público [Vídeo Views] [ABO]</t>
   </si>
   <si>
-    <t>ACTIVE</t>
+    <t>PAUSED</t>
   </si>
   <si>
     <t>OUTCOME_ENGAGEMENT</t>
@@ -75,7 +75,7 @@
     <t>31/03/2026</t>
   </si>
   <si>
-    <t>✅ Ativa</t>
+    <t>⏸️ Pausada</t>
   </si>
   <si>
     <t>120244701890430204</t>
@@ -96,13 +96,7 @@
     <t>[Syra] PÁGINA DE CAPTURA [Cadastro] [CBO]</t>
   </si>
   <si>
-    <t>PAUSED</t>
-  </si>
-  <si>
     <t>25/02/2026</t>
-  </si>
-  <si>
-    <t>⏸️ Pausada</t>
   </si>
   <si>
     <t>120243510129130204</t>
@@ -284,7 +278,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -299,11 +293,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -324,7 +313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -335,7 +324,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -842,8 +830,8 @@
       <c r="B4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>27</v>
+      <c r="C4" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>23</v>
@@ -852,7 +840,7 @@
         <v>20</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G4" s="6">
         <v>0</v>
@@ -879,18 +867,18 @@
         <v>0</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D5" t="s">
         <v>23</v>
@@ -899,7 +887,7 @@
         <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -926,27 +914,27 @@
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>33</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>35</v>
       </c>
       <c r="E6" s="8">
         <v>10</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G6" s="6">
         <v>0</v>
@@ -973,18 +961,18 @@
         <v>0</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>27</v>
+        <v>36</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -993,7 +981,7 @@
         <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1020,18 +1008,18 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>27</v>
+        <v>38</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>23</v>
@@ -1040,7 +1028,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G8" s="6">
         <v>0</v>
@@ -1067,18 +1055,18 @@
         <v>0</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>27</v>
+        <v>41</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D9" t="s">
         <v>23</v>
@@ -1087,7 +1075,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -1114,18 +1102,18 @@
         <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>27</v>
+        <v>44</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>18</v>
@@ -1134,7 +1122,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G10" s="6">
         <v>0</v>
@@ -1161,18 +1149,18 @@
         <v>0</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>27</v>
+        <v>47</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D11" t="s">
         <v>18</v>
@@ -1181,7 +1169,7 @@
         <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1208,18 +1196,18 @@
         <v>0</v>
       </c>
       <c r="O11" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>27</v>
+        <v>50</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>23</v>
@@ -1228,7 +1216,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G12" s="6">
         <v>0</v>
@@ -1255,18 +1243,18 @@
         <v>0</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>27</v>
+        <v>53</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D13" t="s">
         <v>23</v>
@@ -1275,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -1302,18 +1290,18 @@
         <v>0</v>
       </c>
       <c r="O13" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>27</v>
+        <v>56</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>23</v>
@@ -1322,7 +1310,7 @@
         <v>25</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G14" s="6">
         <v>0</v>
@@ -1349,18 +1337,18 @@
         <v>0</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>27</v>
+        <v>59</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D15" t="s">
         <v>23</v>
@@ -1369,7 +1357,7 @@
         <v>40</v>
       </c>
       <c r="F15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -1396,18 +1384,18 @@
         <v>0</v>
       </c>
       <c r="O15" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>27</v>
+        <v>61</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>23</v>
@@ -1416,7 +1404,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G16" s="6">
         <v>0</v>
@@ -1443,18 +1431,18 @@
         <v>0</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>27</v>
+        <v>63</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D17" t="s">
         <v>23</v>
@@ -1463,7 +1451,7 @@
         <v>20</v>
       </c>
       <c r="F17" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -1490,18 +1478,18 @@
         <v>0</v>
       </c>
       <c r="O17" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>27</v>
+        <v>66</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>18</v>
@@ -1510,7 +1498,7 @@
         <v>10</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G18" s="6">
         <v>0</v>
@@ -1537,7 +1525,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1566,13 +1554,13 @@
   <sheetData>
     <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -1581,7 +1569,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
@@ -1596,30 +1584,30 @@
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" t="s">
         <v>75</v>
       </c>
-      <c r="B2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" t="s">
-        <v>77</v>
-      </c>
       <c r="D2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1637,7 +1625,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1664,19 +1652,19 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -1694,24 +1682,24 @@
         <v>2</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1726,10 +1714,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>